<commit_message>
Reset Excel Table for CNC3X-08
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-08.xlsx
+++ b/FM-MN-07_CNC3X-08.xlsx
@@ -1804,45 +1804,37 @@
           <t>Worm up เครื่องจักร 15 นาที ทุกครั้งที่ใช้งาน</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n"/>
-      <c r="D6" s="22" t="n"/>
-      <c r="E6" s="22" t="n"/>
-      <c r="F6" s="22" t="n"/>
-      <c r="G6" s="22" t="n"/>
-      <c r="H6" s="22" t="n"/>
-      <c r="I6" s="22" t="n"/>
-      <c r="J6" s="22" t="n"/>
-      <c r="K6" s="22" t="n"/>
-      <c r="L6" s="22" t="n"/>
-      <c r="M6" s="22" t="n"/>
-      <c r="N6" s="22" t="n"/>
-      <c r="O6" s="22" t="n"/>
-      <c r="P6" s="22" t="n"/>
-      <c r="Q6" s="22" t="n"/>
-      <c r="R6" s="22" t="n"/>
-      <c r="S6" s="22" t="n"/>
-      <c r="T6" s="22" t="n"/>
-      <c r="U6" s="22" t="n"/>
-      <c r="V6" s="22" t="n"/>
-      <c r="W6" s="22" t="n"/>
-      <c r="X6" s="22" t="n"/>
-      <c r="Y6" s="23" t="n"/>
-      <c r="Z6" s="22" t="n"/>
-      <c r="AA6" s="23" t="n"/>
-      <c r="AB6" s="22" t="n"/>
-      <c r="AC6" s="22" t="n"/>
-      <c r="AD6" s="22" t="n"/>
-      <c r="AE6" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF6" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG6" s="22" t="n"/>
+      <c r="C6" s="22" t="inlineStr"/>
+      <c r="D6" s="22" t="inlineStr"/>
+      <c r="E6" s="22" t="inlineStr"/>
+      <c r="F6" s="22" t="inlineStr"/>
+      <c r="G6" s="22" t="inlineStr"/>
+      <c r="H6" s="22" t="inlineStr"/>
+      <c r="I6" s="22" t="inlineStr"/>
+      <c r="J6" s="22" t="inlineStr"/>
+      <c r="K6" s="22" t="inlineStr"/>
+      <c r="L6" s="22" t="inlineStr"/>
+      <c r="M6" s="22" t="inlineStr"/>
+      <c r="N6" s="22" t="inlineStr"/>
+      <c r="O6" s="22" t="inlineStr"/>
+      <c r="P6" s="22" t="inlineStr"/>
+      <c r="Q6" s="22" t="inlineStr"/>
+      <c r="R6" s="22" t="inlineStr"/>
+      <c r="S6" s="22" t="inlineStr"/>
+      <c r="T6" s="22" t="inlineStr"/>
+      <c r="U6" s="22" t="inlineStr"/>
+      <c r="V6" s="22" t="inlineStr"/>
+      <c r="W6" s="22" t="inlineStr"/>
+      <c r="X6" s="22" t="inlineStr"/>
+      <c r="Y6" s="23" t="inlineStr"/>
+      <c r="Z6" s="22" t="inlineStr"/>
+      <c r="AA6" s="23" t="inlineStr"/>
+      <c r="AB6" s="22" t="inlineStr"/>
+      <c r="AC6" s="22" t="inlineStr"/>
+      <c r="AD6" s="22" t="inlineStr"/>
+      <c r="AE6" s="23" t="inlineStr"/>
+      <c r="AF6" s="23" t="inlineStr"/>
+      <c r="AG6" s="22" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="14" t="n">
@@ -1853,45 +1845,37 @@
           <t>เช็คระดับนำมันที่ Pump Hydraulic ทุกวัน เติมเมื่อพร่อง</t>
         </is>
       </c>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="n"/>
-      <c r="K7" s="22" t="n"/>
-      <c r="L7" s="22" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="22" t="n"/>
-      <c r="O7" s="22" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
-      <c r="T7" s="22" t="n"/>
-      <c r="U7" s="22" t="n"/>
-      <c r="V7" s="22" t="n"/>
-      <c r="W7" s="22" t="n"/>
-      <c r="X7" s="22" t="n"/>
-      <c r="Y7" s="23" t="n"/>
-      <c r="Z7" s="22" t="n"/>
-      <c r="AA7" s="23" t="n"/>
-      <c r="AB7" s="22" t="n"/>
-      <c r="AC7" s="22" t="n"/>
-      <c r="AD7" s="22" t="n"/>
-      <c r="AE7" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF7" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG7" s="22" t="n"/>
+      <c r="C7" s="22" t="inlineStr"/>
+      <c r="D7" s="22" t="inlineStr"/>
+      <c r="E7" s="22" t="inlineStr"/>
+      <c r="F7" s="22" t="inlineStr"/>
+      <c r="G7" s="22" t="inlineStr"/>
+      <c r="H7" s="22" t="inlineStr"/>
+      <c r="I7" s="22" t="inlineStr"/>
+      <c r="J7" s="22" t="inlineStr"/>
+      <c r="K7" s="22" t="inlineStr"/>
+      <c r="L7" s="22" t="inlineStr"/>
+      <c r="M7" s="22" t="inlineStr"/>
+      <c r="N7" s="22" t="inlineStr"/>
+      <c r="O7" s="22" t="inlineStr"/>
+      <c r="P7" s="22" t="inlineStr"/>
+      <c r="Q7" s="22" t="inlineStr"/>
+      <c r="R7" s="22" t="inlineStr"/>
+      <c r="S7" s="22" t="inlineStr"/>
+      <c r="T7" s="22" t="inlineStr"/>
+      <c r="U7" s="22" t="inlineStr"/>
+      <c r="V7" s="22" t="inlineStr"/>
+      <c r="W7" s="22" t="inlineStr"/>
+      <c r="X7" s="22" t="inlineStr"/>
+      <c r="Y7" s="23" t="inlineStr"/>
+      <c r="Z7" s="22" t="inlineStr"/>
+      <c r="AA7" s="23" t="inlineStr"/>
+      <c r="AB7" s="22" t="inlineStr"/>
+      <c r="AC7" s="22" t="inlineStr"/>
+      <c r="AD7" s="22" t="inlineStr"/>
+      <c r="AE7" s="23" t="inlineStr"/>
+      <c r="AF7" s="23" t="inlineStr"/>
+      <c r="AG7" s="22" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="14" t="n">
@@ -1902,45 +1886,37 @@
           <t>ทำความสะอาด Air filter Mesh ทุกวัน</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
-      <c r="F8" s="22" t="n"/>
-      <c r="G8" s="22" t="n"/>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="22" t="n"/>
-      <c r="J8" s="22" t="n"/>
-      <c r="K8" s="22" t="n"/>
-      <c r="L8" s="22" t="n"/>
-      <c r="M8" s="22" t="n"/>
-      <c r="N8" s="22" t="n"/>
-      <c r="O8" s="22" t="n"/>
-      <c r="P8" s="22" t="n"/>
-      <c r="Q8" s="22" t="n"/>
-      <c r="R8" s="22" t="n"/>
-      <c r="S8" s="22" t="n"/>
-      <c r="T8" s="22" t="n"/>
-      <c r="U8" s="22" t="n"/>
-      <c r="V8" s="22" t="n"/>
-      <c r="W8" s="22" t="n"/>
-      <c r="X8" s="22" t="n"/>
-      <c r="Y8" s="23" t="n"/>
-      <c r="Z8" s="22" t="n"/>
-      <c r="AA8" s="23" t="n"/>
-      <c r="AB8" s="22" t="n"/>
-      <c r="AC8" s="22" t="n"/>
-      <c r="AD8" s="22" t="n"/>
-      <c r="AE8" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF8" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG8" s="22" t="n"/>
+      <c r="C8" s="22" t="inlineStr"/>
+      <c r="D8" s="22" t="inlineStr"/>
+      <c r="E8" s="22" t="inlineStr"/>
+      <c r="F8" s="22" t="inlineStr"/>
+      <c r="G8" s="22" t="inlineStr"/>
+      <c r="H8" s="22" t="inlineStr"/>
+      <c r="I8" s="22" t="inlineStr"/>
+      <c r="J8" s="22" t="inlineStr"/>
+      <c r="K8" s="22" t="inlineStr"/>
+      <c r="L8" s="22" t="inlineStr"/>
+      <c r="M8" s="22" t="inlineStr"/>
+      <c r="N8" s="22" t="inlineStr"/>
+      <c r="O8" s="22" t="inlineStr"/>
+      <c r="P8" s="22" t="inlineStr"/>
+      <c r="Q8" s="22" t="inlineStr"/>
+      <c r="R8" s="22" t="inlineStr"/>
+      <c r="S8" s="22" t="inlineStr"/>
+      <c r="T8" s="22" t="inlineStr"/>
+      <c r="U8" s="22" t="inlineStr"/>
+      <c r="V8" s="22" t="inlineStr"/>
+      <c r="W8" s="22" t="inlineStr"/>
+      <c r="X8" s="22" t="inlineStr"/>
+      <c r="Y8" s="23" t="inlineStr"/>
+      <c r="Z8" s="22" t="inlineStr"/>
+      <c r="AA8" s="23" t="inlineStr"/>
+      <c r="AB8" s="22" t="inlineStr"/>
+      <c r="AC8" s="22" t="inlineStr"/>
+      <c r="AD8" s="22" t="inlineStr"/>
+      <c r="AE8" s="23" t="inlineStr"/>
+      <c r="AF8" s="23" t="inlineStr"/>
+      <c r="AG8" s="22" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="14" t="n">
@@ -1951,45 +1927,37 @@
           <t>ตรวจเช็คแรงดัน Air Control Unit ปกติเฉลี่ยที่ 0.5 Mpa</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="22" t="n"/>
-      <c r="F9" s="22" t="n"/>
-      <c r="G9" s="22" t="n"/>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="22" t="n"/>
-      <c r="J9" s="22" t="n"/>
-      <c r="K9" s="22" t="n"/>
-      <c r="L9" s="22" t="n"/>
-      <c r="M9" s="22" t="n"/>
-      <c r="N9" s="22" t="n"/>
-      <c r="O9" s="22" t="n"/>
-      <c r="P9" s="22" t="n"/>
-      <c r="Q9" s="22" t="n"/>
-      <c r="R9" s="22" t="n"/>
-      <c r="S9" s="22" t="n"/>
-      <c r="T9" s="22" t="n"/>
-      <c r="U9" s="22" t="n"/>
-      <c r="V9" s="22" t="n"/>
-      <c r="W9" s="22" t="n"/>
-      <c r="X9" s="22" t="n"/>
-      <c r="Y9" s="23" t="n"/>
-      <c r="Z9" s="22" t="n"/>
-      <c r="AA9" s="23" t="n"/>
-      <c r="AB9" s="22" t="n"/>
-      <c r="AC9" s="22" t="n"/>
-      <c r="AD9" s="22" t="n"/>
-      <c r="AE9" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF9" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG9" s="22" t="n"/>
+      <c r="C9" s="22" t="inlineStr"/>
+      <c r="D9" s="22" t="inlineStr"/>
+      <c r="E9" s="22" t="inlineStr"/>
+      <c r="F9" s="22" t="inlineStr"/>
+      <c r="G9" s="22" t="inlineStr"/>
+      <c r="H9" s="22" t="inlineStr"/>
+      <c r="I9" s="22" t="inlineStr"/>
+      <c r="J9" s="22" t="inlineStr"/>
+      <c r="K9" s="22" t="inlineStr"/>
+      <c r="L9" s="22" t="inlineStr"/>
+      <c r="M9" s="22" t="inlineStr"/>
+      <c r="N9" s="22" t="inlineStr"/>
+      <c r="O9" s="22" t="inlineStr"/>
+      <c r="P9" s="22" t="inlineStr"/>
+      <c r="Q9" s="22" t="inlineStr"/>
+      <c r="R9" s="22" t="inlineStr"/>
+      <c r="S9" s="22" t="inlineStr"/>
+      <c r="T9" s="22" t="inlineStr"/>
+      <c r="U9" s="22" t="inlineStr"/>
+      <c r="V9" s="22" t="inlineStr"/>
+      <c r="W9" s="22" t="inlineStr"/>
+      <c r="X9" s="22" t="inlineStr"/>
+      <c r="Y9" s="23" t="inlineStr"/>
+      <c r="Z9" s="22" t="inlineStr"/>
+      <c r="AA9" s="23" t="inlineStr"/>
+      <c r="AB9" s="22" t="inlineStr"/>
+      <c r="AC9" s="22" t="inlineStr"/>
+      <c r="AD9" s="22" t="inlineStr"/>
+      <c r="AE9" s="23" t="inlineStr"/>
+      <c r="AF9" s="23" t="inlineStr"/>
+      <c r="AG9" s="22" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="14" t="n">
@@ -2000,45 +1968,37 @@
           <t>เช็คน้ำมันชุด Gear ของ ATC ทุกวัน(เปลี่ยนถ่ายทุกปี)</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="22" t="n"/>
-      <c r="E10" s="22" t="n"/>
-      <c r="F10" s="22" t="n"/>
-      <c r="G10" s="22" t="n"/>
-      <c r="H10" s="22" t="n"/>
-      <c r="I10" s="22" t="n"/>
-      <c r="J10" s="22" t="n"/>
-      <c r="K10" s="22" t="n"/>
-      <c r="L10" s="22" t="n"/>
-      <c r="M10" s="22" t="n"/>
-      <c r="N10" s="22" t="n"/>
-      <c r="O10" s="22" t="n"/>
-      <c r="P10" s="22" t="n"/>
-      <c r="Q10" s="22" t="n"/>
-      <c r="R10" s="22" t="n"/>
-      <c r="S10" s="22" t="n"/>
-      <c r="T10" s="22" t="n"/>
-      <c r="U10" s="22" t="n"/>
-      <c r="V10" s="22" t="n"/>
-      <c r="W10" s="22" t="n"/>
-      <c r="X10" s="22" t="n"/>
-      <c r="Y10" s="23" t="n"/>
-      <c r="Z10" s="22" t="n"/>
-      <c r="AA10" s="23" t="n"/>
-      <c r="AB10" s="22" t="n"/>
-      <c r="AC10" s="22" t="n"/>
-      <c r="AD10" s="22" t="n"/>
-      <c r="AE10" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF10" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG10" s="22" t="n"/>
+      <c r="C10" s="22" t="inlineStr"/>
+      <c r="D10" s="22" t="inlineStr"/>
+      <c r="E10" s="22" t="inlineStr"/>
+      <c r="F10" s="22" t="inlineStr"/>
+      <c r="G10" s="22" t="inlineStr"/>
+      <c r="H10" s="22" t="inlineStr"/>
+      <c r="I10" s="22" t="inlineStr"/>
+      <c r="J10" s="22" t="inlineStr"/>
+      <c r="K10" s="22" t="inlineStr"/>
+      <c r="L10" s="22" t="inlineStr"/>
+      <c r="M10" s="22" t="inlineStr"/>
+      <c r="N10" s="22" t="inlineStr"/>
+      <c r="O10" s="22" t="inlineStr"/>
+      <c r="P10" s="22" t="inlineStr"/>
+      <c r="Q10" s="22" t="inlineStr"/>
+      <c r="R10" s="22" t="inlineStr"/>
+      <c r="S10" s="22" t="inlineStr"/>
+      <c r="T10" s="22" t="inlineStr"/>
+      <c r="U10" s="22" t="inlineStr"/>
+      <c r="V10" s="22" t="inlineStr"/>
+      <c r="W10" s="22" t="inlineStr"/>
+      <c r="X10" s="22" t="inlineStr"/>
+      <c r="Y10" s="23" t="inlineStr"/>
+      <c r="Z10" s="22" t="inlineStr"/>
+      <c r="AA10" s="23" t="inlineStr"/>
+      <c r="AB10" s="22" t="inlineStr"/>
+      <c r="AC10" s="22" t="inlineStr"/>
+      <c r="AD10" s="22" t="inlineStr"/>
+      <c r="AE10" s="23" t="inlineStr"/>
+      <c r="AF10" s="23" t="inlineStr"/>
+      <c r="AG10" s="22" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="14" t="n">
@@ -2049,45 +2009,37 @@
           <t>อัดจารบี Ballscrew และ Linear Guideทุก 1ครั้งต่อเดือน</t>
         </is>
       </c>
-      <c r="C11" s="22" t="n"/>
-      <c r="D11" s="22" t="n"/>
-      <c r="E11" s="22" t="n"/>
-      <c r="F11" s="22" t="n"/>
-      <c r="G11" s="22" t="n"/>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="22" t="n"/>
-      <c r="J11" s="22" t="n"/>
-      <c r="K11" s="22" t="n"/>
-      <c r="L11" s="22" t="n"/>
-      <c r="M11" s="22" t="n"/>
-      <c r="N11" s="22" t="n"/>
-      <c r="O11" s="22" t="n"/>
-      <c r="P11" s="22" t="n"/>
-      <c r="Q11" s="22" t="n"/>
-      <c r="R11" s="22" t="n"/>
-      <c r="S11" s="22" t="n"/>
-      <c r="T11" s="22" t="n"/>
-      <c r="U11" s="22" t="n"/>
-      <c r="V11" s="22" t="n"/>
-      <c r="W11" s="22" t="n"/>
-      <c r="X11" s="22" t="n"/>
-      <c r="Y11" s="23" t="n"/>
-      <c r="Z11" s="22" t="n"/>
-      <c r="AA11" s="23" t="n"/>
-      <c r="AB11" s="22" t="n"/>
-      <c r="AC11" s="22" t="n"/>
-      <c r="AD11" s="22" t="n"/>
-      <c r="AE11" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF11" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG11" s="22" t="n"/>
+      <c r="C11" s="22" t="inlineStr"/>
+      <c r="D11" s="22" t="inlineStr"/>
+      <c r="E11" s="22" t="inlineStr"/>
+      <c r="F11" s="22" t="inlineStr"/>
+      <c r="G11" s="22" t="inlineStr"/>
+      <c r="H11" s="22" t="inlineStr"/>
+      <c r="I11" s="22" t="inlineStr"/>
+      <c r="J11" s="22" t="inlineStr"/>
+      <c r="K11" s="22" t="inlineStr"/>
+      <c r="L11" s="22" t="inlineStr"/>
+      <c r="M11" s="22" t="inlineStr"/>
+      <c r="N11" s="22" t="inlineStr"/>
+      <c r="O11" s="22" t="inlineStr"/>
+      <c r="P11" s="22" t="inlineStr"/>
+      <c r="Q11" s="22" t="inlineStr"/>
+      <c r="R11" s="22" t="inlineStr"/>
+      <c r="S11" s="22" t="inlineStr"/>
+      <c r="T11" s="22" t="inlineStr"/>
+      <c r="U11" s="22" t="inlineStr"/>
+      <c r="V11" s="22" t="inlineStr"/>
+      <c r="W11" s="22" t="inlineStr"/>
+      <c r="X11" s="22" t="inlineStr"/>
+      <c r="Y11" s="23" t="inlineStr"/>
+      <c r="Z11" s="22" t="inlineStr"/>
+      <c r="AA11" s="23" t="inlineStr"/>
+      <c r="AB11" s="22" t="inlineStr"/>
+      <c r="AC11" s="22" t="inlineStr"/>
+      <c r="AD11" s="22" t="inlineStr"/>
+      <c r="AE11" s="23" t="inlineStr"/>
+      <c r="AF11" s="23" t="inlineStr"/>
+      <c r="AG11" s="22" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="14" t="n">
@@ -2098,45 +2050,37 @@
           <t>ตรวจสอบการเคลื่อนที่ของแกนทุกแกน (X,Y,Z)</t>
         </is>
       </c>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="22" t="n"/>
-      <c r="I12" s="22" t="n"/>
-      <c r="J12" s="22" t="n"/>
-      <c r="K12" s="22" t="n"/>
-      <c r="L12" s="22" t="n"/>
-      <c r="M12" s="22" t="n"/>
-      <c r="N12" s="22" t="n"/>
-      <c r="O12" s="22" t="n"/>
-      <c r="P12" s="22" t="n"/>
-      <c r="Q12" s="22" t="n"/>
-      <c r="R12" s="22" t="n"/>
-      <c r="S12" s="22" t="n"/>
-      <c r="T12" s="22" t="n"/>
-      <c r="U12" s="22" t="n"/>
-      <c r="V12" s="22" t="n"/>
-      <c r="W12" s="22" t="n"/>
-      <c r="X12" s="22" t="n"/>
-      <c r="Y12" s="23" t="n"/>
-      <c r="Z12" s="22" t="n"/>
-      <c r="AA12" s="23" t="n"/>
-      <c r="AB12" s="22" t="n"/>
-      <c r="AC12" s="22" t="n"/>
-      <c r="AD12" s="22" t="n"/>
-      <c r="AE12" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF12" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG12" s="22" t="n"/>
+      <c r="C12" s="22" t="inlineStr"/>
+      <c r="D12" s="22" t="inlineStr"/>
+      <c r="E12" s="22" t="inlineStr"/>
+      <c r="F12" s="22" t="inlineStr"/>
+      <c r="G12" s="22" t="inlineStr"/>
+      <c r="H12" s="22" t="inlineStr"/>
+      <c r="I12" s="22" t="inlineStr"/>
+      <c r="J12" s="22" t="inlineStr"/>
+      <c r="K12" s="22" t="inlineStr"/>
+      <c r="L12" s="22" t="inlineStr"/>
+      <c r="M12" s="22" t="inlineStr"/>
+      <c r="N12" s="22" t="inlineStr"/>
+      <c r="O12" s="22" t="inlineStr"/>
+      <c r="P12" s="22" t="inlineStr"/>
+      <c r="Q12" s="22" t="inlineStr"/>
+      <c r="R12" s="22" t="inlineStr"/>
+      <c r="S12" s="22" t="inlineStr"/>
+      <c r="T12" s="22" t="inlineStr"/>
+      <c r="U12" s="22" t="inlineStr"/>
+      <c r="V12" s="22" t="inlineStr"/>
+      <c r="W12" s="22" t="inlineStr"/>
+      <c r="X12" s="22" t="inlineStr"/>
+      <c r="Y12" s="23" t="inlineStr"/>
+      <c r="Z12" s="22" t="inlineStr"/>
+      <c r="AA12" s="23" t="inlineStr"/>
+      <c r="AB12" s="22" t="inlineStr"/>
+      <c r="AC12" s="22" t="inlineStr"/>
+      <c r="AD12" s="22" t="inlineStr"/>
+      <c r="AE12" s="23" t="inlineStr"/>
+      <c r="AF12" s="23" t="inlineStr"/>
+      <c r="AG12" s="22" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="14" t="n">
@@ -2147,45 +2091,37 @@
           <t>ตรวจสอบสภาพของน้ำ Coolant ถ่ายรูปค่าที่วัดได้ส่งเข้าระบบ</t>
         </is>
       </c>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="22" t="n"/>
-      <c r="J13" s="22" t="n"/>
-      <c r="K13" s="22" t="n"/>
-      <c r="L13" s="22" t="n"/>
-      <c r="M13" s="22" t="n"/>
-      <c r="N13" s="22" t="n"/>
-      <c r="O13" s="22" t="n"/>
-      <c r="P13" s="22" t="n"/>
-      <c r="Q13" s="22" t="n"/>
-      <c r="R13" s="22" t="n"/>
-      <c r="S13" s="22" t="n"/>
-      <c r="T13" s="22" t="n"/>
-      <c r="U13" s="22" t="n"/>
-      <c r="V13" s="22" t="n"/>
-      <c r="W13" s="22" t="n"/>
-      <c r="X13" s="22" t="n"/>
-      <c r="Y13" s="23" t="n"/>
-      <c r="Z13" s="22" t="n"/>
-      <c r="AA13" s="23" t="n"/>
-      <c r="AB13" s="22" t="n"/>
-      <c r="AC13" s="22" t="n"/>
-      <c r="AD13" s="22" t="n"/>
-      <c r="AE13" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF13" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG13" s="22" t="n"/>
+      <c r="C13" s="22" t="inlineStr"/>
+      <c r="D13" s="22" t="inlineStr"/>
+      <c r="E13" s="22" t="inlineStr"/>
+      <c r="F13" s="22" t="inlineStr"/>
+      <c r="G13" s="22" t="inlineStr"/>
+      <c r="H13" s="22" t="inlineStr"/>
+      <c r="I13" s="22" t="inlineStr"/>
+      <c r="J13" s="22" t="inlineStr"/>
+      <c r="K13" s="22" t="inlineStr"/>
+      <c r="L13" s="22" t="inlineStr"/>
+      <c r="M13" s="22" t="inlineStr"/>
+      <c r="N13" s="22" t="inlineStr"/>
+      <c r="O13" s="22" t="inlineStr"/>
+      <c r="P13" s="22" t="inlineStr"/>
+      <c r="Q13" s="22" t="inlineStr"/>
+      <c r="R13" s="22" t="inlineStr"/>
+      <c r="S13" s="22" t="inlineStr"/>
+      <c r="T13" s="22" t="inlineStr"/>
+      <c r="U13" s="22" t="inlineStr"/>
+      <c r="V13" s="22" t="inlineStr"/>
+      <c r="W13" s="22" t="inlineStr"/>
+      <c r="X13" s="22" t="inlineStr"/>
+      <c r="Y13" s="23" t="inlineStr"/>
+      <c r="Z13" s="22" t="inlineStr"/>
+      <c r="AA13" s="23" t="inlineStr"/>
+      <c r="AB13" s="22" t="inlineStr"/>
+      <c r="AC13" s="22" t="inlineStr"/>
+      <c r="AD13" s="22" t="inlineStr"/>
+      <c r="AE13" s="23" t="inlineStr"/>
+      <c r="AF13" s="23" t="inlineStr"/>
+      <c r="AG13" s="22" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="14" t="n">
@@ -2196,45 +2132,37 @@
           <t>การทำงานของ Coolant pump</t>
         </is>
       </c>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
-      <c r="I14" s="22" t="n"/>
-      <c r="J14" s="22" t="n"/>
-      <c r="K14" s="22" t="n"/>
-      <c r="L14" s="22" t="n"/>
-      <c r="M14" s="22" t="n"/>
-      <c r="N14" s="22" t="n"/>
-      <c r="O14" s="22" t="n"/>
-      <c r="P14" s="22" t="n"/>
-      <c r="Q14" s="22" t="n"/>
-      <c r="R14" s="22" t="n"/>
-      <c r="S14" s="22" t="n"/>
-      <c r="T14" s="22" t="n"/>
-      <c r="U14" s="22" t="n"/>
-      <c r="V14" s="22" t="n"/>
-      <c r="W14" s="22" t="n"/>
-      <c r="X14" s="22" t="n"/>
-      <c r="Y14" s="23" t="n"/>
-      <c r="Z14" s="22" t="n"/>
-      <c r="AA14" s="23" t="n"/>
-      <c r="AB14" s="22" t="n"/>
-      <c r="AC14" s="22" t="n"/>
-      <c r="AD14" s="22" t="n"/>
-      <c r="AE14" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF14" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG14" s="22" t="n"/>
+      <c r="C14" s="22" t="inlineStr"/>
+      <c r="D14" s="22" t="inlineStr"/>
+      <c r="E14" s="22" t="inlineStr"/>
+      <c r="F14" s="22" t="inlineStr"/>
+      <c r="G14" s="22" t="inlineStr"/>
+      <c r="H14" s="22" t="inlineStr"/>
+      <c r="I14" s="22" t="inlineStr"/>
+      <c r="J14" s="22" t="inlineStr"/>
+      <c r="K14" s="22" t="inlineStr"/>
+      <c r="L14" s="22" t="inlineStr"/>
+      <c r="M14" s="22" t="inlineStr"/>
+      <c r="N14" s="22" t="inlineStr"/>
+      <c r="O14" s="22" t="inlineStr"/>
+      <c r="P14" s="22" t="inlineStr"/>
+      <c r="Q14" s="22" t="inlineStr"/>
+      <c r="R14" s="22" t="inlineStr"/>
+      <c r="S14" s="22" t="inlineStr"/>
+      <c r="T14" s="22" t="inlineStr"/>
+      <c r="U14" s="22" t="inlineStr"/>
+      <c r="V14" s="22" t="inlineStr"/>
+      <c r="W14" s="22" t="inlineStr"/>
+      <c r="X14" s="22" t="inlineStr"/>
+      <c r="Y14" s="23" t="inlineStr"/>
+      <c r="Z14" s="22" t="inlineStr"/>
+      <c r="AA14" s="23" t="inlineStr"/>
+      <c r="AB14" s="22" t="inlineStr"/>
+      <c r="AC14" s="22" t="inlineStr"/>
+      <c r="AD14" s="22" t="inlineStr"/>
+      <c r="AE14" s="23" t="inlineStr"/>
+      <c r="AF14" s="23" t="inlineStr"/>
+      <c r="AG14" s="22" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="14" t="n">
@@ -2245,45 +2173,37 @@
           <t>การทำงานของ Unclamp และการเปลี่ยน Tool</t>
         </is>
       </c>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="22" t="n"/>
-      <c r="J15" s="22" t="n"/>
-      <c r="K15" s="22" t="n"/>
-      <c r="L15" s="22" t="n"/>
-      <c r="M15" s="22" t="n"/>
-      <c r="N15" s="22" t="n"/>
-      <c r="O15" s="22" t="n"/>
-      <c r="P15" s="22" t="n"/>
-      <c r="Q15" s="22" t="n"/>
-      <c r="R15" s="22" t="n"/>
-      <c r="S15" s="22" t="n"/>
-      <c r="T15" s="22" t="n"/>
-      <c r="U15" s="22" t="n"/>
-      <c r="V15" s="22" t="n"/>
-      <c r="W15" s="22" t="n"/>
-      <c r="X15" s="22" t="n"/>
-      <c r="Y15" s="23" t="n"/>
-      <c r="Z15" s="22" t="n"/>
-      <c r="AA15" s="23" t="n"/>
-      <c r="AB15" s="22" t="n"/>
-      <c r="AC15" s="22" t="n"/>
-      <c r="AD15" s="22" t="n"/>
-      <c r="AE15" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF15" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG15" s="22" t="n"/>
+      <c r="C15" s="22" t="inlineStr"/>
+      <c r="D15" s="22" t="inlineStr"/>
+      <c r="E15" s="22" t="inlineStr"/>
+      <c r="F15" s="22" t="inlineStr"/>
+      <c r="G15" s="22" t="inlineStr"/>
+      <c r="H15" s="22" t="inlineStr"/>
+      <c r="I15" s="22" t="inlineStr"/>
+      <c r="J15" s="22" t="inlineStr"/>
+      <c r="K15" s="22" t="inlineStr"/>
+      <c r="L15" s="22" t="inlineStr"/>
+      <c r="M15" s="22" t="inlineStr"/>
+      <c r="N15" s="22" t="inlineStr"/>
+      <c r="O15" s="22" t="inlineStr"/>
+      <c r="P15" s="22" t="inlineStr"/>
+      <c r="Q15" s="22" t="inlineStr"/>
+      <c r="R15" s="22" t="inlineStr"/>
+      <c r="S15" s="22" t="inlineStr"/>
+      <c r="T15" s="22" t="inlineStr"/>
+      <c r="U15" s="22" t="inlineStr"/>
+      <c r="V15" s="22" t="inlineStr"/>
+      <c r="W15" s="22" t="inlineStr"/>
+      <c r="X15" s="22" t="inlineStr"/>
+      <c r="Y15" s="23" t="inlineStr"/>
+      <c r="Z15" s="22" t="inlineStr"/>
+      <c r="AA15" s="23" t="inlineStr"/>
+      <c r="AB15" s="22" t="inlineStr"/>
+      <c r="AC15" s="22" t="inlineStr"/>
+      <c r="AD15" s="22" t="inlineStr"/>
+      <c r="AE15" s="23" t="inlineStr"/>
+      <c r="AF15" s="23" t="inlineStr"/>
+      <c r="AG15" s="22" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="14" t="n">
@@ -2294,45 +2214,37 @@
           <t>การทำงานของ Spindle</t>
         </is>
       </c>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="22" t="n"/>
-      <c r="F16" s="22" t="n"/>
-      <c r="G16" s="22" t="n"/>
-      <c r="H16" s="22" t="n"/>
-      <c r="I16" s="22" t="n"/>
-      <c r="J16" s="22" t="n"/>
-      <c r="K16" s="22" t="n"/>
-      <c r="L16" s="22" t="n"/>
-      <c r="M16" s="22" t="n"/>
-      <c r="N16" s="22" t="n"/>
-      <c r="O16" s="22" t="n"/>
-      <c r="P16" s="22" t="n"/>
-      <c r="Q16" s="22" t="n"/>
-      <c r="R16" s="22" t="n"/>
-      <c r="S16" s="22" t="n"/>
-      <c r="T16" s="22" t="n"/>
-      <c r="U16" s="22" t="n"/>
-      <c r="V16" s="22" t="n"/>
-      <c r="W16" s="22" t="n"/>
-      <c r="X16" s="22" t="n"/>
-      <c r="Y16" s="23" t="n"/>
-      <c r="Z16" s="22" t="n"/>
-      <c r="AA16" s="23" t="n"/>
-      <c r="AB16" s="22" t="n"/>
-      <c r="AC16" s="22" t="n"/>
-      <c r="AD16" s="22" t="n"/>
-      <c r="AE16" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF16" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG16" s="22" t="n"/>
+      <c r="C16" s="22" t="inlineStr"/>
+      <c r="D16" s="22" t="inlineStr"/>
+      <c r="E16" s="22" t="inlineStr"/>
+      <c r="F16" s="22" t="inlineStr"/>
+      <c r="G16" s="22" t="inlineStr"/>
+      <c r="H16" s="22" t="inlineStr"/>
+      <c r="I16" s="22" t="inlineStr"/>
+      <c r="J16" s="22" t="inlineStr"/>
+      <c r="K16" s="22" t="inlineStr"/>
+      <c r="L16" s="22" t="inlineStr"/>
+      <c r="M16" s="22" t="inlineStr"/>
+      <c r="N16" s="22" t="inlineStr"/>
+      <c r="O16" s="22" t="inlineStr"/>
+      <c r="P16" s="22" t="inlineStr"/>
+      <c r="Q16" s="22" t="inlineStr"/>
+      <c r="R16" s="22" t="inlineStr"/>
+      <c r="S16" s="22" t="inlineStr"/>
+      <c r="T16" s="22" t="inlineStr"/>
+      <c r="U16" s="22" t="inlineStr"/>
+      <c r="V16" s="22" t="inlineStr"/>
+      <c r="W16" s="22" t="inlineStr"/>
+      <c r="X16" s="22" t="inlineStr"/>
+      <c r="Y16" s="23" t="inlineStr"/>
+      <c r="Z16" s="22" t="inlineStr"/>
+      <c r="AA16" s="23" t="inlineStr"/>
+      <c r="AB16" s="22" t="inlineStr"/>
+      <c r="AC16" s="22" t="inlineStr"/>
+      <c r="AD16" s="22" t="inlineStr"/>
+      <c r="AE16" s="23" t="inlineStr"/>
+      <c r="AF16" s="23" t="inlineStr"/>
+      <c r="AG16" s="22" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="14" t="n">
@@ -2343,45 +2255,37 @@
           <t>การทำงานของ Arm เปลี่ยน Tool</t>
         </is>
       </c>
-      <c r="C17" s="22" t="n"/>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="22" t="n"/>
-      <c r="F17" s="22" t="n"/>
-      <c r="G17" s="22" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="22" t="n"/>
-      <c r="J17" s="22" t="n"/>
-      <c r="K17" s="22" t="n"/>
-      <c r="L17" s="22" t="n"/>
-      <c r="M17" s="22" t="n"/>
-      <c r="N17" s="22" t="n"/>
-      <c r="O17" s="22" t="n"/>
-      <c r="P17" s="22" t="n"/>
-      <c r="Q17" s="22" t="n"/>
-      <c r="R17" s="22" t="n"/>
-      <c r="S17" s="22" t="n"/>
-      <c r="T17" s="22" t="n"/>
-      <c r="U17" s="22" t="n"/>
-      <c r="V17" s="22" t="n"/>
-      <c r="W17" s="22" t="n"/>
-      <c r="X17" s="22" t="n"/>
-      <c r="Y17" s="23" t="n"/>
-      <c r="Z17" s="22" t="n"/>
-      <c r="AA17" s="23" t="n"/>
-      <c r="AB17" s="22" t="n"/>
-      <c r="AC17" s="22" t="n"/>
-      <c r="AD17" s="22" t="n"/>
-      <c r="AE17" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF17" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG17" s="22" t="n"/>
+      <c r="C17" s="22" t="inlineStr"/>
+      <c r="D17" s="22" t="inlineStr"/>
+      <c r="E17" s="22" t="inlineStr"/>
+      <c r="F17" s="22" t="inlineStr"/>
+      <c r="G17" s="22" t="inlineStr"/>
+      <c r="H17" s="22" t="inlineStr"/>
+      <c r="I17" s="22" t="inlineStr"/>
+      <c r="J17" s="22" t="inlineStr"/>
+      <c r="K17" s="22" t="inlineStr"/>
+      <c r="L17" s="22" t="inlineStr"/>
+      <c r="M17" s="22" t="inlineStr"/>
+      <c r="N17" s="22" t="inlineStr"/>
+      <c r="O17" s="22" t="inlineStr"/>
+      <c r="P17" s="22" t="inlineStr"/>
+      <c r="Q17" s="22" t="inlineStr"/>
+      <c r="R17" s="22" t="inlineStr"/>
+      <c r="S17" s="22" t="inlineStr"/>
+      <c r="T17" s="22" t="inlineStr"/>
+      <c r="U17" s="22" t="inlineStr"/>
+      <c r="V17" s="22" t="inlineStr"/>
+      <c r="W17" s="22" t="inlineStr"/>
+      <c r="X17" s="22" t="inlineStr"/>
+      <c r="Y17" s="23" t="inlineStr"/>
+      <c r="Z17" s="22" t="inlineStr"/>
+      <c r="AA17" s="23" t="inlineStr"/>
+      <c r="AB17" s="22" t="inlineStr"/>
+      <c r="AC17" s="22" t="inlineStr"/>
+      <c r="AD17" s="22" t="inlineStr"/>
+      <c r="AE17" s="23" t="inlineStr"/>
+      <c r="AF17" s="23" t="inlineStr"/>
+      <c r="AG17" s="22" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="14" t="n">
@@ -2392,45 +2296,37 @@
           <t>ตรวจสอบระดับของน้ำ Coolant เติมเมื่ออยู่ระดับที่ต่ำ</t>
         </is>
       </c>
-      <c r="C18" s="22" t="n"/>
-      <c r="D18" s="22" t="n"/>
-      <c r="E18" s="22" t="n"/>
-      <c r="F18" s="22" t="n"/>
-      <c r="G18" s="22" t="n"/>
-      <c r="H18" s="22" t="n"/>
-      <c r="I18" s="22" t="n"/>
-      <c r="J18" s="22" t="n"/>
-      <c r="K18" s="22" t="n"/>
-      <c r="L18" s="22" t="n"/>
-      <c r="M18" s="22" t="n"/>
-      <c r="N18" s="22" t="n"/>
-      <c r="O18" s="22" t="n"/>
-      <c r="P18" s="22" t="n"/>
-      <c r="Q18" s="22" t="n"/>
-      <c r="R18" s="22" t="n"/>
-      <c r="S18" s="22" t="n"/>
-      <c r="T18" s="22" t="n"/>
-      <c r="U18" s="22" t="n"/>
-      <c r="V18" s="22" t="n"/>
-      <c r="W18" s="22" t="n"/>
-      <c r="X18" s="22" t="n"/>
-      <c r="Y18" s="23" t="n"/>
-      <c r="Z18" s="22" t="n"/>
-      <c r="AA18" s="23" t="n"/>
-      <c r="AB18" s="22" t="n"/>
-      <c r="AC18" s="22" t="n"/>
-      <c r="AD18" s="22" t="n"/>
-      <c r="AE18" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF18" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG18" s="22" t="n"/>
+      <c r="C18" s="22" t="inlineStr"/>
+      <c r="D18" s="22" t="inlineStr"/>
+      <c r="E18" s="22" t="inlineStr"/>
+      <c r="F18" s="22" t="inlineStr"/>
+      <c r="G18" s="22" t="inlineStr"/>
+      <c r="H18" s="22" t="inlineStr"/>
+      <c r="I18" s="22" t="inlineStr"/>
+      <c r="J18" s="22" t="inlineStr"/>
+      <c r="K18" s="22" t="inlineStr"/>
+      <c r="L18" s="22" t="inlineStr"/>
+      <c r="M18" s="22" t="inlineStr"/>
+      <c r="N18" s="22" t="inlineStr"/>
+      <c r="O18" s="22" t="inlineStr"/>
+      <c r="P18" s="22" t="inlineStr"/>
+      <c r="Q18" s="22" t="inlineStr"/>
+      <c r="R18" s="22" t="inlineStr"/>
+      <c r="S18" s="22" t="inlineStr"/>
+      <c r="T18" s="22" t="inlineStr"/>
+      <c r="U18" s="22" t="inlineStr"/>
+      <c r="V18" s="22" t="inlineStr"/>
+      <c r="W18" s="22" t="inlineStr"/>
+      <c r="X18" s="22" t="inlineStr"/>
+      <c r="Y18" s="23" t="inlineStr"/>
+      <c r="Z18" s="22" t="inlineStr"/>
+      <c r="AA18" s="23" t="inlineStr"/>
+      <c r="AB18" s="22" t="inlineStr"/>
+      <c r="AC18" s="22" t="inlineStr"/>
+      <c r="AD18" s="22" t="inlineStr"/>
+      <c r="AE18" s="23" t="inlineStr"/>
+      <c r="AF18" s="23" t="inlineStr"/>
+      <c r="AG18" s="22" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="14" t="n">
@@ -2441,45 +2337,37 @@
           <t>ความสะอาดทั่วไปของเครื่องจักรโดยรวม</t>
         </is>
       </c>
-      <c r="C19" s="22" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="22" t="n"/>
-      <c r="F19" s="22" t="n"/>
-      <c r="G19" s="22" t="n"/>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="22" t="n"/>
-      <c r="J19" s="22" t="n"/>
-      <c r="K19" s="22" t="n"/>
-      <c r="L19" s="22" t="n"/>
-      <c r="M19" s="22" t="n"/>
-      <c r="N19" s="22" t="n"/>
-      <c r="O19" s="22" t="n"/>
-      <c r="P19" s="22" t="n"/>
-      <c r="Q19" s="22" t="n"/>
-      <c r="R19" s="22" t="n"/>
-      <c r="S19" s="22" t="n"/>
-      <c r="T19" s="22" t="n"/>
-      <c r="U19" s="22" t="n"/>
-      <c r="V19" s="22" t="n"/>
-      <c r="W19" s="22" t="n"/>
-      <c r="X19" s="22" t="n"/>
-      <c r="Y19" s="23" t="n"/>
-      <c r="Z19" s="22" t="n"/>
-      <c r="AA19" s="23" t="n"/>
-      <c r="AB19" s="22" t="n"/>
-      <c r="AC19" s="22" t="n"/>
-      <c r="AD19" s="22" t="n"/>
-      <c r="AE19" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF19" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG19" s="22" t="n"/>
+      <c r="C19" s="22" t="inlineStr"/>
+      <c r="D19" s="22" t="inlineStr"/>
+      <c r="E19" s="22" t="inlineStr"/>
+      <c r="F19" s="22" t="inlineStr"/>
+      <c r="G19" s="22" t="inlineStr"/>
+      <c r="H19" s="22" t="inlineStr"/>
+      <c r="I19" s="22" t="inlineStr"/>
+      <c r="J19" s="22" t="inlineStr"/>
+      <c r="K19" s="22" t="inlineStr"/>
+      <c r="L19" s="22" t="inlineStr"/>
+      <c r="M19" s="22" t="inlineStr"/>
+      <c r="N19" s="22" t="inlineStr"/>
+      <c r="O19" s="22" t="inlineStr"/>
+      <c r="P19" s="22" t="inlineStr"/>
+      <c r="Q19" s="22" t="inlineStr"/>
+      <c r="R19" s="22" t="inlineStr"/>
+      <c r="S19" s="22" t="inlineStr"/>
+      <c r="T19" s="22" t="inlineStr"/>
+      <c r="U19" s="22" t="inlineStr"/>
+      <c r="V19" s="22" t="inlineStr"/>
+      <c r="W19" s="22" t="inlineStr"/>
+      <c r="X19" s="22" t="inlineStr"/>
+      <c r="Y19" s="23" t="inlineStr"/>
+      <c r="Z19" s="22" t="inlineStr"/>
+      <c r="AA19" s="23" t="inlineStr"/>
+      <c r="AB19" s="22" t="inlineStr"/>
+      <c r="AC19" s="22" t="inlineStr"/>
+      <c r="AD19" s="22" t="inlineStr"/>
+      <c r="AE19" s="23" t="inlineStr"/>
+      <c r="AF19" s="23" t="inlineStr"/>
+      <c r="AG19" s="22" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="14" t="n">
@@ -2490,45 +2378,37 @@
           <t>ตรวจสอบความพร้อมสภาพโดยรวม(ฟังด้วยหู ดูด้วยตา)</t>
         </is>
       </c>
-      <c r="C20" s="22" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="22" t="n"/>
-      <c r="G20" s="22" t="n"/>
-      <c r="H20" s="22" t="n"/>
-      <c r="I20" s="22" t="n"/>
-      <c r="J20" s="22" t="n"/>
-      <c r="K20" s="22" t="n"/>
-      <c r="L20" s="22" t="n"/>
-      <c r="M20" s="22" t="n"/>
-      <c r="N20" s="22" t="n"/>
-      <c r="O20" s="22" t="n"/>
-      <c r="P20" s="22" t="n"/>
-      <c r="Q20" s="22" t="n"/>
-      <c r="R20" s="22" t="n"/>
-      <c r="S20" s="22" t="n"/>
-      <c r="T20" s="22" t="n"/>
-      <c r="U20" s="22" t="n"/>
-      <c r="V20" s="22" t="n"/>
-      <c r="W20" s="22" t="n"/>
-      <c r="X20" s="22" t="n"/>
-      <c r="Y20" s="23" t="n"/>
-      <c r="Z20" s="22" t="n"/>
-      <c r="AA20" s="23" t="n"/>
-      <c r="AB20" s="22" t="n"/>
-      <c r="AC20" s="22" t="n"/>
-      <c r="AD20" s="22" t="n"/>
-      <c r="AE20" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF20" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG20" s="22" t="n"/>
+      <c r="C20" s="22" t="inlineStr"/>
+      <c r="D20" s="22" t="inlineStr"/>
+      <c r="E20" s="22" t="inlineStr"/>
+      <c r="F20" s="22" t="inlineStr"/>
+      <c r="G20" s="22" t="inlineStr"/>
+      <c r="H20" s="22" t="inlineStr"/>
+      <c r="I20" s="22" t="inlineStr"/>
+      <c r="J20" s="22" t="inlineStr"/>
+      <c r="K20" s="22" t="inlineStr"/>
+      <c r="L20" s="22" t="inlineStr"/>
+      <c r="M20" s="22" t="inlineStr"/>
+      <c r="N20" s="22" t="inlineStr"/>
+      <c r="O20" s="22" t="inlineStr"/>
+      <c r="P20" s="22" t="inlineStr"/>
+      <c r="Q20" s="22" t="inlineStr"/>
+      <c r="R20" s="22" t="inlineStr"/>
+      <c r="S20" s="22" t="inlineStr"/>
+      <c r="T20" s="22" t="inlineStr"/>
+      <c r="U20" s="22" t="inlineStr"/>
+      <c r="V20" s="22" t="inlineStr"/>
+      <c r="W20" s="22" t="inlineStr"/>
+      <c r="X20" s="22" t="inlineStr"/>
+      <c r="Y20" s="23" t="inlineStr"/>
+      <c r="Z20" s="22" t="inlineStr"/>
+      <c r="AA20" s="23" t="inlineStr"/>
+      <c r="AB20" s="22" t="inlineStr"/>
+      <c r="AC20" s="22" t="inlineStr"/>
+      <c r="AD20" s="22" t="inlineStr"/>
+      <c r="AE20" s="23" t="inlineStr"/>
+      <c r="AF20" s="23" t="inlineStr"/>
+      <c r="AG20" s="22" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="15" t="n">
@@ -2539,88 +2419,72 @@
           <t>ตรวจสอบสายไฮโดรลิกส์ และสายลม</t>
         </is>
       </c>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="22" t="n"/>
-      <c r="F21" s="22" t="n"/>
-      <c r="G21" s="22" t="n"/>
-      <c r="H21" s="22" t="n"/>
-      <c r="I21" s="22" t="n"/>
-      <c r="J21" s="22" t="n"/>
-      <c r="K21" s="22" t="n"/>
-      <c r="L21" s="22" t="n"/>
-      <c r="M21" s="22" t="n"/>
-      <c r="N21" s="22" t="n"/>
-      <c r="O21" s="22" t="n"/>
-      <c r="P21" s="22" t="n"/>
-      <c r="Q21" s="22" t="n"/>
-      <c r="R21" s="22" t="n"/>
-      <c r="S21" s="22" t="n"/>
-      <c r="T21" s="22" t="n"/>
-      <c r="U21" s="22" t="n"/>
-      <c r="V21" s="22" t="n"/>
-      <c r="W21" s="22" t="n"/>
-      <c r="X21" s="22" t="n"/>
-      <c r="Y21" s="23" t="n"/>
-      <c r="Z21" s="22" t="n"/>
-      <c r="AA21" s="23" t="n"/>
-      <c r="AB21" s="22" t="n"/>
-      <c r="AC21" s="22" t="n"/>
-      <c r="AD21" s="22" t="n"/>
-      <c r="AE21" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF21" s="23" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AG21" s="22" t="n"/>
+      <c r="C21" s="22" t="inlineStr"/>
+      <c r="D21" s="22" t="inlineStr"/>
+      <c r="E21" s="22" t="inlineStr"/>
+      <c r="F21" s="22" t="inlineStr"/>
+      <c r="G21" s="22" t="inlineStr"/>
+      <c r="H21" s="22" t="inlineStr"/>
+      <c r="I21" s="22" t="inlineStr"/>
+      <c r="J21" s="22" t="inlineStr"/>
+      <c r="K21" s="22" t="inlineStr"/>
+      <c r="L21" s="22" t="inlineStr"/>
+      <c r="M21" s="22" t="inlineStr"/>
+      <c r="N21" s="22" t="inlineStr"/>
+      <c r="O21" s="22" t="inlineStr"/>
+      <c r="P21" s="22" t="inlineStr"/>
+      <c r="Q21" s="22" t="inlineStr"/>
+      <c r="R21" s="22" t="inlineStr"/>
+      <c r="S21" s="22" t="inlineStr"/>
+      <c r="T21" s="22" t="inlineStr"/>
+      <c r="U21" s="22" t="inlineStr"/>
+      <c r="V21" s="22" t="inlineStr"/>
+      <c r="W21" s="22" t="inlineStr"/>
+      <c r="X21" s="22" t="inlineStr"/>
+      <c r="Y21" s="23" t="inlineStr"/>
+      <c r="Z21" s="22" t="inlineStr"/>
+      <c r="AA21" s="23" t="inlineStr"/>
+      <c r="AB21" s="22" t="inlineStr"/>
+      <c r="AC21" s="22" t="inlineStr"/>
+      <c r="AD21" s="22" t="inlineStr"/>
+      <c r="AE21" s="23" t="inlineStr"/>
+      <c r="AF21" s="23" t="inlineStr"/>
+      <c r="AG21" s="22" t="inlineStr"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="8" t="n"/>
-      <c r="C22" s="30" t="n"/>
-      <c r="D22" s="30" t="n"/>
-      <c r="E22" s="30" t="n"/>
-      <c r="F22" s="30" t="n"/>
-      <c r="G22" s="30" t="n"/>
-      <c r="H22" s="30" t="n"/>
-      <c r="I22" s="30" t="n"/>
-      <c r="J22" s="30" t="n"/>
-      <c r="K22" s="30" t="n"/>
-      <c r="L22" s="30" t="n"/>
-      <c r="M22" s="30" t="n"/>
-      <c r="N22" s="30" t="n"/>
-      <c r="O22" s="30" t="n"/>
-      <c r="P22" s="30" t="n"/>
-      <c r="Q22" s="30" t="n"/>
-      <c r="R22" s="30" t="n"/>
-      <c r="S22" s="30" t="n"/>
-      <c r="T22" s="30" t="n"/>
-      <c r="U22" s="30" t="n"/>
-      <c r="V22" s="30" t="n"/>
-      <c r="W22" s="30" t="n"/>
-      <c r="X22" s="32" t="n"/>
-      <c r="Y22" s="32" t="n"/>
-      <c r="Z22" s="30" t="n"/>
-      <c r="AA22" s="32" t="n"/>
-      <c r="AB22" s="30" t="n"/>
-      <c r="AC22" s="30" t="n"/>
-      <c r="AD22" s="30" t="n"/>
-      <c r="AE22" s="32" t="inlineStr">
-        <is>
-          <t>ณัฐพงศ์</t>
-        </is>
-      </c>
-      <c r="AF22" s="32" t="inlineStr">
-        <is>
-          <t>ณัฐพงศ์</t>
-        </is>
-      </c>
-      <c r="AG22" s="30" t="n"/>
+      <c r="C22" s="30" t="inlineStr"/>
+      <c r="D22" s="30" t="inlineStr"/>
+      <c r="E22" s="30" t="inlineStr"/>
+      <c r="F22" s="30" t="inlineStr"/>
+      <c r="G22" s="30" t="inlineStr"/>
+      <c r="H22" s="30" t="inlineStr"/>
+      <c r="I22" s="30" t="inlineStr"/>
+      <c r="J22" s="30" t="inlineStr"/>
+      <c r="K22" s="30" t="inlineStr"/>
+      <c r="L22" s="30" t="inlineStr"/>
+      <c r="M22" s="30" t="inlineStr"/>
+      <c r="N22" s="30" t="inlineStr"/>
+      <c r="O22" s="30" t="inlineStr"/>
+      <c r="P22" s="30" t="inlineStr"/>
+      <c r="Q22" s="30" t="inlineStr"/>
+      <c r="R22" s="30" t="inlineStr"/>
+      <c r="S22" s="30" t="inlineStr"/>
+      <c r="T22" s="30" t="inlineStr"/>
+      <c r="U22" s="30" t="inlineStr"/>
+      <c r="V22" s="30" t="inlineStr"/>
+      <c r="W22" s="30" t="inlineStr"/>
+      <c r="X22" s="32" t="inlineStr"/>
+      <c r="Y22" s="32" t="inlineStr"/>
+      <c r="Z22" s="30" t="inlineStr"/>
+      <c r="AA22" s="32" t="inlineStr"/>
+      <c r="AB22" s="30" t="inlineStr"/>
+      <c r="AC22" s="30" t="inlineStr"/>
+      <c r="AD22" s="30" t="inlineStr"/>
+      <c r="AE22" s="32" t="inlineStr"/>
+      <c r="AF22" s="32" t="inlineStr"/>
+      <c r="AG22" s="30" t="inlineStr"/>
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="B23" s="9" t="n"/>
@@ -2658,37 +2522,37 @@
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="B24" s="9" t="n"/>
-      <c r="C24" s="26" t="n"/>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="26" t="n"/>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="26" t="n"/>
-      <c r="H24" s="26" t="n"/>
-      <c r="I24" s="26" t="n"/>
-      <c r="J24" s="26" t="n"/>
-      <c r="K24" s="26" t="n"/>
-      <c r="L24" s="26" t="n"/>
-      <c r="M24" s="26" t="n"/>
-      <c r="N24" s="26" t="n"/>
-      <c r="O24" s="26" t="n"/>
-      <c r="P24" s="26" t="n"/>
-      <c r="Q24" s="26" t="n"/>
-      <c r="R24" s="26" t="n"/>
-      <c r="S24" s="26" t="n"/>
-      <c r="T24" s="26" t="n"/>
-      <c r="U24" s="26" t="n"/>
-      <c r="V24" s="26" t="n"/>
-      <c r="W24" s="26" t="n"/>
-      <c r="X24" s="31" t="n"/>
-      <c r="Y24" s="31" t="n"/>
-      <c r="Z24" s="26" t="n"/>
-      <c r="AA24" s="31" t="n"/>
-      <c r="AB24" s="26" t="n"/>
-      <c r="AC24" s="26" t="n"/>
-      <c r="AD24" s="26" t="n"/>
-      <c r="AE24" s="26" t="n"/>
-      <c r="AF24" s="26" t="n"/>
-      <c r="AG24" s="26" t="n"/>
+      <c r="C24" s="26" t="inlineStr"/>
+      <c r="D24" s="26" t="inlineStr"/>
+      <c r="E24" s="26" t="inlineStr"/>
+      <c r="F24" s="26" t="inlineStr"/>
+      <c r="G24" s="26" t="inlineStr"/>
+      <c r="H24" s="26" t="inlineStr"/>
+      <c r="I24" s="26" t="inlineStr"/>
+      <c r="J24" s="26" t="inlineStr"/>
+      <c r="K24" s="26" t="inlineStr"/>
+      <c r="L24" s="26" t="inlineStr"/>
+      <c r="M24" s="26" t="inlineStr"/>
+      <c r="N24" s="26" t="inlineStr"/>
+      <c r="O24" s="26" t="inlineStr"/>
+      <c r="P24" s="26" t="inlineStr"/>
+      <c r="Q24" s="26" t="inlineStr"/>
+      <c r="R24" s="26" t="inlineStr"/>
+      <c r="S24" s="26" t="inlineStr"/>
+      <c r="T24" s="26" t="inlineStr"/>
+      <c r="U24" s="26" t="inlineStr"/>
+      <c r="V24" s="26" t="inlineStr"/>
+      <c r="W24" s="26" t="inlineStr"/>
+      <c r="X24" s="31" t="inlineStr"/>
+      <c r="Y24" s="31" t="inlineStr"/>
+      <c r="Z24" s="26" t="inlineStr"/>
+      <c r="AA24" s="31" t="inlineStr"/>
+      <c r="AB24" s="26" t="inlineStr"/>
+      <c r="AC24" s="26" t="inlineStr"/>
+      <c r="AD24" s="26" t="inlineStr"/>
+      <c r="AE24" s="26" t="inlineStr"/>
+      <c r="AF24" s="26" t="inlineStr"/>
+      <c r="AG24" s="26" t="inlineStr"/>
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="B25" s="9" t="n"/>
@@ -2735,11 +2599,7 @@
       <c r="Y27" s="21" t="n"/>
     </row>
     <row r="28" ht="173.25" customHeight="1">
-      <c r="B28" s="46" t="inlineStr">
-        <is>
-          <t>[วันที่ 29]: บอร์ดคลูลิ่งเสีย ตอนนี้ต่อตรงอยู่,  [วันที่ 30]: บอร์ดคลูลิ่งเสีย ตอนนี้ต่อตรงอยู่, บอร์ดคูลิ่งเสีย</t>
-        </is>
-      </c>
+      <c r="B28" s="46" t="inlineStr"/>
     </row>
     <row r="29" ht="21" customHeight="1">
       <c r="AA29" s="19" t="n"/>

</xml_diff>

<commit_message>
Direct Write Excel for CNC3X-08 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-08.xlsx
+++ b/FM-MN-07_CNC3X-08.xlsx
@@ -1809,7 +1809,11 @@
       <c r="E6" s="22" t="inlineStr"/>
       <c r="F6" s="22" t="inlineStr"/>
       <c r="G6" s="22" t="inlineStr"/>
-      <c r="H6" s="22" t="inlineStr"/>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="22" t="inlineStr"/>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
@@ -1850,7 +1854,11 @@
       <c r="E7" s="22" t="inlineStr"/>
       <c r="F7" s="22" t="inlineStr"/>
       <c r="G7" s="22" t="inlineStr"/>
-      <c r="H7" s="22" t="inlineStr"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="22" t="inlineStr"/>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
@@ -1891,7 +1899,11 @@
       <c r="E8" s="22" t="inlineStr"/>
       <c r="F8" s="22" t="inlineStr"/>
       <c r="G8" s="22" t="inlineStr"/>
-      <c r="H8" s="22" t="inlineStr"/>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="22" t="inlineStr"/>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
@@ -1932,7 +1944,11 @@
       <c r="E9" s="22" t="inlineStr"/>
       <c r="F9" s="22" t="inlineStr"/>
       <c r="G9" s="22" t="inlineStr"/>
-      <c r="H9" s="22" t="inlineStr"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="22" t="inlineStr"/>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
@@ -1973,7 +1989,11 @@
       <c r="E10" s="22" t="inlineStr"/>
       <c r="F10" s="22" t="inlineStr"/>
       <c r="G10" s="22" t="inlineStr"/>
-      <c r="H10" s="22" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="22" t="inlineStr"/>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
@@ -2014,7 +2034,11 @@
       <c r="E11" s="22" t="inlineStr"/>
       <c r="F11" s="22" t="inlineStr"/>
       <c r="G11" s="22" t="inlineStr"/>
-      <c r="H11" s="22" t="inlineStr"/>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I11" s="22" t="inlineStr"/>
       <c r="J11" s="22" t="inlineStr"/>
       <c r="K11" s="22" t="inlineStr"/>
@@ -2055,7 +2079,11 @@
       <c r="E12" s="22" t="inlineStr"/>
       <c r="F12" s="22" t="inlineStr"/>
       <c r="G12" s="22" t="inlineStr"/>
-      <c r="H12" s="22" t="inlineStr"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="22" t="inlineStr"/>
       <c r="J12" s="22" t="inlineStr"/>
       <c r="K12" s="22" t="inlineStr"/>
@@ -2096,7 +2124,11 @@
       <c r="E13" s="22" t="inlineStr"/>
       <c r="F13" s="22" t="inlineStr"/>
       <c r="G13" s="22" t="inlineStr"/>
-      <c r="H13" s="22" t="inlineStr"/>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="22" t="inlineStr"/>
       <c r="J13" s="22" t="inlineStr"/>
       <c r="K13" s="22" t="inlineStr"/>
@@ -2137,7 +2169,11 @@
       <c r="E14" s="22" t="inlineStr"/>
       <c r="F14" s="22" t="inlineStr"/>
       <c r="G14" s="22" t="inlineStr"/>
-      <c r="H14" s="22" t="inlineStr"/>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I14" s="22" t="inlineStr"/>
       <c r="J14" s="22" t="inlineStr"/>
       <c r="K14" s="22" t="inlineStr"/>
@@ -2178,7 +2214,11 @@
       <c r="E15" s="22" t="inlineStr"/>
       <c r="F15" s="22" t="inlineStr"/>
       <c r="G15" s="22" t="inlineStr"/>
-      <c r="H15" s="22" t="inlineStr"/>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I15" s="22" t="inlineStr"/>
       <c r="J15" s="22" t="inlineStr"/>
       <c r="K15" s="22" t="inlineStr"/>
@@ -2219,7 +2259,11 @@
       <c r="E16" s="22" t="inlineStr"/>
       <c r="F16" s="22" t="inlineStr"/>
       <c r="G16" s="22" t="inlineStr"/>
-      <c r="H16" s="22" t="inlineStr"/>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I16" s="22" t="inlineStr"/>
       <c r="J16" s="22" t="inlineStr"/>
       <c r="K16" s="22" t="inlineStr"/>
@@ -2260,7 +2304,11 @@
       <c r="E17" s="22" t="inlineStr"/>
       <c r="F17" s="22" t="inlineStr"/>
       <c r="G17" s="22" t="inlineStr"/>
-      <c r="H17" s="22" t="inlineStr"/>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I17" s="22" t="inlineStr"/>
       <c r="J17" s="22" t="inlineStr"/>
       <c r="K17" s="22" t="inlineStr"/>
@@ -2301,7 +2349,11 @@
       <c r="E18" s="22" t="inlineStr"/>
       <c r="F18" s="22" t="inlineStr"/>
       <c r="G18" s="22" t="inlineStr"/>
-      <c r="H18" s="22" t="inlineStr"/>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I18" s="22" t="inlineStr"/>
       <c r="J18" s="22" t="inlineStr"/>
       <c r="K18" s="22" t="inlineStr"/>
@@ -2342,7 +2394,11 @@
       <c r="E19" s="22" t="inlineStr"/>
       <c r="F19" s="22" t="inlineStr"/>
       <c r="G19" s="22" t="inlineStr"/>
-      <c r="H19" s="22" t="inlineStr"/>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I19" s="22" t="inlineStr"/>
       <c r="J19" s="22" t="inlineStr"/>
       <c r="K19" s="22" t="inlineStr"/>
@@ -2383,7 +2439,11 @@
       <c r="E20" s="22" t="inlineStr"/>
       <c r="F20" s="22" t="inlineStr"/>
       <c r="G20" s="22" t="inlineStr"/>
-      <c r="H20" s="22" t="inlineStr"/>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I20" s="22" t="inlineStr"/>
       <c r="J20" s="22" t="inlineStr"/>
       <c r="K20" s="22" t="inlineStr"/>
@@ -2424,7 +2484,11 @@
       <c r="E21" s="22" t="inlineStr"/>
       <c r="F21" s="22" t="inlineStr"/>
       <c r="G21" s="22" t="inlineStr"/>
-      <c r="H21" s="22" t="inlineStr"/>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I21" s="22" t="inlineStr"/>
       <c r="J21" s="22" t="inlineStr"/>
       <c r="K21" s="22" t="inlineStr"/>
@@ -2459,7 +2523,11 @@
       <c r="E22" s="30" t="inlineStr"/>
       <c r="F22" s="30" t="inlineStr"/>
       <c r="G22" s="30" t="inlineStr"/>
-      <c r="H22" s="30" t="inlineStr"/>
+      <c r="H22" s="32" t="inlineStr">
+        <is>
+          <t>ณัฐพงศ์</t>
+        </is>
+      </c>
       <c r="I22" s="30" t="inlineStr"/>
       <c r="J22" s="30" t="inlineStr"/>
       <c r="K22" s="30" t="inlineStr"/>
@@ -2599,7 +2667,11 @@
       <c r="Y27" s="21" t="n"/>
     </row>
     <row r="28" ht="173.25" customHeight="1">
-      <c r="B28" s="46" t="inlineStr"/>
+      <c r="B28" s="46" t="inlineStr">
+        <is>
+          <t>[วันที่ 6]: ข้อ 3: บอร์ดคลูลิ่งเสีย</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="21" customHeight="1">
       <c r="AA29" s="19" t="n"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-08 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-08.xlsx
+++ b/FM-MN-07_CNC3X-08.xlsx
@@ -1814,7 +1814,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr"/>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
       <c r="L6" s="22" t="inlineStr"/>
@@ -1859,7 +1863,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="22" t="inlineStr"/>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr"/>
@@ -1904,7 +1912,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr"/>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
       <c r="L8" s="22" t="inlineStr"/>
@@ -1949,7 +1961,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="22" t="inlineStr"/>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
       <c r="L9" s="22" t="inlineStr"/>
@@ -1994,7 +2010,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr"/>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
       <c r="L10" s="22" t="inlineStr"/>
@@ -2039,7 +2059,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I11" s="22" t="inlineStr"/>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J11" s="22" t="inlineStr"/>
       <c r="K11" s="22" t="inlineStr"/>
       <c r="L11" s="22" t="inlineStr"/>
@@ -2084,7 +2108,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="22" t="inlineStr"/>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="22" t="inlineStr"/>
       <c r="K12" s="22" t="inlineStr"/>
       <c r="L12" s="22" t="inlineStr"/>
@@ -2129,7 +2157,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I13" s="22" t="inlineStr"/>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J13" s="22" t="inlineStr"/>
       <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="22" t="inlineStr"/>
@@ -2174,7 +2206,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I14" s="22" t="inlineStr"/>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J14" s="22" t="inlineStr"/>
       <c r="K14" s="22" t="inlineStr"/>
       <c r="L14" s="22" t="inlineStr"/>
@@ -2219,7 +2255,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I15" s="22" t="inlineStr"/>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J15" s="22" t="inlineStr"/>
       <c r="K15" s="22" t="inlineStr"/>
       <c r="L15" s="22" t="inlineStr"/>
@@ -2264,7 +2304,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I16" s="22" t="inlineStr"/>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J16" s="22" t="inlineStr"/>
       <c r="K16" s="22" t="inlineStr"/>
       <c r="L16" s="22" t="inlineStr"/>
@@ -2309,7 +2353,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I17" s="22" t="inlineStr"/>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="inlineStr"/>
       <c r="K17" s="22" t="inlineStr"/>
       <c r="L17" s="22" t="inlineStr"/>
@@ -2354,7 +2402,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I18" s="22" t="inlineStr"/>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J18" s="22" t="inlineStr"/>
       <c r="K18" s="22" t="inlineStr"/>
       <c r="L18" s="22" t="inlineStr"/>
@@ -2399,7 +2451,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I19" s="22" t="inlineStr"/>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="inlineStr"/>
       <c r="K19" s="22" t="inlineStr"/>
       <c r="L19" s="22" t="inlineStr"/>
@@ -2444,7 +2500,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I20" s="22" t="inlineStr"/>
+      <c r="I20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J20" s="22" t="inlineStr"/>
       <c r="K20" s="22" t="inlineStr"/>
       <c r="L20" s="22" t="inlineStr"/>
@@ -2489,7 +2549,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I21" s="22" t="inlineStr"/>
+      <c r="I21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J21" s="22" t="inlineStr"/>
       <c r="K21" s="22" t="inlineStr"/>
       <c r="L21" s="22" t="inlineStr"/>
@@ -2528,7 +2592,11 @@
           <t>ณัฐพงศ์</t>
         </is>
       </c>
-      <c r="I22" s="30" t="inlineStr"/>
+      <c r="I22" s="32" t="inlineStr">
+        <is>
+          <t>ณัฐพงศ์</t>
+        </is>
+      </c>
       <c r="J22" s="30" t="inlineStr"/>
       <c r="K22" s="30" t="inlineStr"/>
       <c r="L22" s="30" t="inlineStr"/>
@@ -2669,7 +2737,7 @@
     <row r="28" ht="173.25" customHeight="1">
       <c r="B28" s="46" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: บอร์ดคลูลิ่งเสีย</t>
+          <t>[วันที่ 6]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 7]: ข้อ 3: บอร์ดคลูลิ่งเสีย</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-08 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-08.xlsx
+++ b/FM-MN-07_CNC3X-08.xlsx
@@ -1819,7 +1819,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="22" t="inlineStr"/>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="22" t="inlineStr"/>
       <c r="L6" s="22" t="inlineStr"/>
       <c r="M6" s="22" t="inlineStr"/>
@@ -1868,7 +1872,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="22" t="inlineStr"/>
+      <c r="J7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="22" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr"/>
       <c r="M7" s="22" t="inlineStr"/>
@@ -1917,7 +1925,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="22" t="inlineStr"/>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="22" t="inlineStr"/>
       <c r="L8" s="22" t="inlineStr"/>
       <c r="M8" s="22" t="inlineStr"/>
@@ -1966,7 +1978,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="22" t="inlineStr"/>
+      <c r="J9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="22" t="inlineStr"/>
       <c r="L9" s="22" t="inlineStr"/>
       <c r="M9" s="22" t="inlineStr"/>
@@ -2015,7 +2031,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="22" t="inlineStr"/>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="22" t="inlineStr"/>
       <c r="L10" s="22" t="inlineStr"/>
       <c r="M10" s="22" t="inlineStr"/>
@@ -2064,7 +2084,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J11" s="22" t="inlineStr"/>
+      <c r="J11" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K11" s="22" t="inlineStr"/>
       <c r="L11" s="22" t="inlineStr"/>
       <c r="M11" s="22" t="inlineStr"/>
@@ -2113,7 +2137,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="22" t="inlineStr"/>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="22" t="inlineStr"/>
       <c r="L12" s="22" t="inlineStr"/>
       <c r="M12" s="22" t="inlineStr"/>
@@ -2162,7 +2190,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J13" s="22" t="inlineStr"/>
+      <c r="J13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="22" t="inlineStr"/>
       <c r="M13" s="22" t="inlineStr"/>
@@ -2211,7 +2243,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J14" s="22" t="inlineStr"/>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K14" s="22" t="inlineStr"/>
       <c r="L14" s="22" t="inlineStr"/>
       <c r="M14" s="22" t="inlineStr"/>
@@ -2260,7 +2296,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J15" s="22" t="inlineStr"/>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K15" s="22" t="inlineStr"/>
       <c r="L15" s="22" t="inlineStr"/>
       <c r="M15" s="22" t="inlineStr"/>
@@ -2309,7 +2349,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J16" s="22" t="inlineStr"/>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K16" s="22" t="inlineStr"/>
       <c r="L16" s="22" t="inlineStr"/>
       <c r="M16" s="22" t="inlineStr"/>
@@ -2358,7 +2402,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J17" s="22" t="inlineStr"/>
+      <c r="J17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K17" s="22" t="inlineStr"/>
       <c r="L17" s="22" t="inlineStr"/>
       <c r="M17" s="22" t="inlineStr"/>
@@ -2407,7 +2455,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J18" s="22" t="inlineStr"/>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K18" s="22" t="inlineStr"/>
       <c r="L18" s="22" t="inlineStr"/>
       <c r="M18" s="22" t="inlineStr"/>
@@ -2456,7 +2508,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J19" s="22" t="inlineStr"/>
+      <c r="J19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K19" s="22" t="inlineStr"/>
       <c r="L19" s="22" t="inlineStr"/>
       <c r="M19" s="22" t="inlineStr"/>
@@ -2505,7 +2561,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J20" s="22" t="inlineStr"/>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K20" s="22" t="inlineStr"/>
       <c r="L20" s="22" t="inlineStr"/>
       <c r="M20" s="22" t="inlineStr"/>
@@ -2554,7 +2614,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J21" s="22" t="inlineStr"/>
+      <c r="J21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K21" s="22" t="inlineStr"/>
       <c r="L21" s="22" t="inlineStr"/>
       <c r="M21" s="22" t="inlineStr"/>
@@ -2597,7 +2661,11 @@
           <t>ณัฐพงศ์</t>
         </is>
       </c>
-      <c r="J22" s="30" t="inlineStr"/>
+      <c r="J22" s="32" t="inlineStr">
+        <is>
+          <t>ณัฐพงศ์</t>
+        </is>
+      </c>
       <c r="K22" s="30" t="inlineStr"/>
       <c r="L22" s="30" t="inlineStr"/>
       <c r="M22" s="30" t="inlineStr"/>
@@ -2741,7 +2809,7 @@
     <row r="28" ht="173.25" customHeight="1">
       <c r="B28" s="46" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 7]: ข้อ 3: บอร์ดคลูลิ่งเสีย</t>
+          <t>[วันที่ 6]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 7]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 8]: ข้อ 3: บอร์ดคูลลิ่งเสีย</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-08 Day 9
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-08.xlsx
+++ b/FM-MN-07_CNC3X-08.xlsx
@@ -1824,7 +1824,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K6" s="22" t="inlineStr"/>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L6" s="22" t="inlineStr"/>
       <c r="M6" s="22" t="inlineStr"/>
       <c r="N6" s="22" t="inlineStr"/>
@@ -1877,7 +1881,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K7" s="22" t="inlineStr"/>
+      <c r="K7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L7" s="22" t="inlineStr"/>
       <c r="M7" s="22" t="inlineStr"/>
       <c r="N7" s="22" t="inlineStr"/>
@@ -1930,7 +1938,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K8" s="22" t="inlineStr"/>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L8" s="22" t="inlineStr"/>
       <c r="M8" s="22" t="inlineStr"/>
       <c r="N8" s="22" t="inlineStr"/>
@@ -1983,7 +1995,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K9" s="22" t="inlineStr"/>
+      <c r="K9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L9" s="22" t="inlineStr"/>
       <c r="M9" s="22" t="inlineStr"/>
       <c r="N9" s="22" t="inlineStr"/>
@@ -2036,7 +2052,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K10" s="22" t="inlineStr"/>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L10" s="22" t="inlineStr"/>
       <c r="M10" s="22" t="inlineStr"/>
       <c r="N10" s="22" t="inlineStr"/>
@@ -2089,7 +2109,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="K11" s="22" t="inlineStr"/>
+      <c r="K11" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L11" s="22" t="inlineStr"/>
       <c r="M11" s="22" t="inlineStr"/>
       <c r="N11" s="22" t="inlineStr"/>
@@ -2142,7 +2166,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K12" s="22" t="inlineStr"/>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L12" s="22" t="inlineStr"/>
       <c r="M12" s="22" t="inlineStr"/>
       <c r="N12" s="22" t="inlineStr"/>
@@ -2195,7 +2223,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K13" s="22" t="inlineStr"/>
+      <c r="K13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L13" s="22" t="inlineStr"/>
       <c r="M13" s="22" t="inlineStr"/>
       <c r="N13" s="22" t="inlineStr"/>
@@ -2248,7 +2280,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K14" s="22" t="inlineStr"/>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L14" s="22" t="inlineStr"/>
       <c r="M14" s="22" t="inlineStr"/>
       <c r="N14" s="22" t="inlineStr"/>
@@ -2301,7 +2337,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K15" s="22" t="inlineStr"/>
+      <c r="K15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L15" s="22" t="inlineStr"/>
       <c r="M15" s="22" t="inlineStr"/>
       <c r="N15" s="22" t="inlineStr"/>
@@ -2354,7 +2394,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K16" s="22" t="inlineStr"/>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L16" s="22" t="inlineStr"/>
       <c r="M16" s="22" t="inlineStr"/>
       <c r="N16" s="22" t="inlineStr"/>
@@ -2407,7 +2451,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K17" s="22" t="inlineStr"/>
+      <c r="K17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L17" s="22" t="inlineStr"/>
       <c r="M17" s="22" t="inlineStr"/>
       <c r="N17" s="22" t="inlineStr"/>
@@ -2460,7 +2508,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K18" s="22" t="inlineStr"/>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L18" s="22" t="inlineStr"/>
       <c r="M18" s="22" t="inlineStr"/>
       <c r="N18" s="22" t="inlineStr"/>
@@ -2513,7 +2565,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K19" s="22" t="inlineStr"/>
+      <c r="K19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L19" s="22" t="inlineStr"/>
       <c r="M19" s="22" t="inlineStr"/>
       <c r="N19" s="22" t="inlineStr"/>
@@ -2566,7 +2622,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K20" s="22" t="inlineStr"/>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L20" s="22" t="inlineStr"/>
       <c r="M20" s="22" t="inlineStr"/>
       <c r="N20" s="22" t="inlineStr"/>
@@ -2619,7 +2679,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="K21" s="22" t="inlineStr"/>
+      <c r="K21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="L21" s="22" t="inlineStr"/>
       <c r="M21" s="22" t="inlineStr"/>
       <c r="N21" s="22" t="inlineStr"/>
@@ -2666,7 +2730,11 @@
           <t>ณัฐพงศ์</t>
         </is>
       </c>
-      <c r="K22" s="30" t="inlineStr"/>
+      <c r="K22" s="32" t="inlineStr">
+        <is>
+          <t>ณัฐพงศ์</t>
+        </is>
+      </c>
       <c r="L22" s="30" t="inlineStr"/>
       <c r="M22" s="30" t="inlineStr"/>
       <c r="N22" s="30" t="inlineStr"/>
@@ -2809,7 +2877,7 @@
     <row r="28" ht="173.25" customHeight="1">
       <c r="B28" s="46" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 7]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 8]: ข้อ 3: บอร์ดคูลลิ่งเสีย</t>
+          <t>[วันที่ 6]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 7]: ข้อ 3: บอร์ดคลูลิ่งเสีย,  [วันที่ 8]: ข้อ 3: บอร์ดคูลลิ่งเสีย,  [วันที่ 9]: ข้อ 3: บอร์ดคลูลิ่งเสีย</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CNC3X-08 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_CNC3X-08.xlsx
+++ b/FM-MN-07_CNC3X-08.xlsx
@@ -1829,7 +1829,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L6" s="22" t="inlineStr"/>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="22" t="inlineStr"/>
       <c r="N6" s="22" t="inlineStr"/>
       <c r="O6" s="22" t="inlineStr"/>
@@ -1886,7 +1890,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L7" s="22" t="inlineStr"/>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="22" t="inlineStr"/>
       <c r="N7" s="22" t="inlineStr"/>
       <c r="O7" s="22" t="inlineStr"/>
@@ -1943,7 +1951,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L8" s="22" t="inlineStr"/>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="22" t="inlineStr"/>
       <c r="N8" s="22" t="inlineStr"/>
       <c r="O8" s="22" t="inlineStr"/>
@@ -2000,7 +2012,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L9" s="22" t="inlineStr"/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="22" t="inlineStr"/>
       <c r="N9" s="22" t="inlineStr"/>
       <c r="O9" s="22" t="inlineStr"/>
@@ -2057,7 +2073,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L10" s="22" t="inlineStr"/>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="22" t="inlineStr"/>
       <c r="N10" s="22" t="inlineStr"/>
       <c r="O10" s="22" t="inlineStr"/>
@@ -2114,7 +2134,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="L11" s="22" t="inlineStr"/>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M11" s="22" t="inlineStr"/>
       <c r="N11" s="22" t="inlineStr"/>
       <c r="O11" s="22" t="inlineStr"/>
@@ -2171,7 +2195,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L12" s="22" t="inlineStr"/>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="22" t="inlineStr"/>
       <c r="N12" s="22" t="inlineStr"/>
       <c r="O12" s="22" t="inlineStr"/>
@@ -2228,7 +2256,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L13" s="22" t="inlineStr"/>
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="22" t="inlineStr"/>
       <c r="N13" s="22" t="inlineStr"/>
       <c r="O13" s="22" t="inlineStr"/>
@@ -2285,7 +2317,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L14" s="22" t="inlineStr"/>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M14" s="22" t="inlineStr"/>
       <c r="N14" s="22" t="inlineStr"/>
       <c r="O14" s="22" t="inlineStr"/>
@@ -2342,7 +2378,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L15" s="22" t="inlineStr"/>
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M15" s="22" t="inlineStr"/>
       <c r="N15" s="22" t="inlineStr"/>
       <c r="O15" s="22" t="inlineStr"/>
@@ -2399,7 +2439,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L16" s="22" t="inlineStr"/>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M16" s="22" t="inlineStr"/>
       <c r="N16" s="22" t="inlineStr"/>
       <c r="O16" s="22" t="inlineStr"/>
@@ -2456,7 +2500,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L17" s="22" t="inlineStr"/>
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M17" s="22" t="inlineStr"/>
       <c r="N17" s="22" t="inlineStr"/>
       <c r="O17" s="22" t="inlineStr"/>
@@ -2513,7 +2561,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L18" s="22" t="inlineStr"/>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M18" s="22" t="inlineStr"/>
       <c r="N18" s="22" t="inlineStr"/>
       <c r="O18" s="22" t="inlineStr"/>
@@ -2570,7 +2622,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L19" s="22" t="inlineStr"/>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M19" s="22" t="inlineStr"/>
       <c r="N19" s="22" t="inlineStr"/>
       <c r="O19" s="22" t="inlineStr"/>
@@ -2627,7 +2683,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L20" s="22" t="inlineStr"/>
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M20" s="22" t="inlineStr"/>
       <c r="N20" s="22" t="inlineStr"/>
       <c r="O20" s="22" t="inlineStr"/>
@@ -2684,7 +2744,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="L21" s="22" t="inlineStr"/>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M21" s="22" t="inlineStr"/>
       <c r="N21" s="22" t="inlineStr"/>
       <c r="O21" s="22" t="inlineStr"/>
@@ -2735,7 +2799,11 @@
           <t>ณัฐพงศ์</t>
         </is>
       </c>
-      <c r="L22" s="30" t="inlineStr"/>
+      <c r="L22" s="32" t="inlineStr">
+        <is>
+          <t>ณัฐพงศ์</t>
+        </is>
+      </c>
       <c r="M22" s="30" t="inlineStr"/>
       <c r="N22" s="30" t="inlineStr"/>
       <c r="O22" s="30" t="inlineStr"/>

</xml_diff>